<commit_message>
create self contained cross-encoder notebook
</commit_message>
<xml_diff>
--- a/Luca/luca_bert_benchmark_results.xlsx
+++ b/Luca/luca_bert_benchmark_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI9"/>
+  <dimension ref="A1:AI10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1461,6 +1461,117 @@
         <v>5.032877683639526</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>a0134a8b2e694bc0823143af5fe5cef4</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Luca</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BERT baseline</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nomic-ai/nomic-embed-text-v1.5</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.3845967905861991</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.3841581004006522</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.5916048288345337</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.5910089015960693</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.2890947659810384</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.2887144883473714</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.3072278499603271</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.3068766593933105</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.3344557285308838</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0.334068775177002</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>2026-05-27 15:10:47</t>
+        </is>
+      </c>
+      <c r="AE10" t="n">
+        <v>3.848027638026646</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>3.958618760108948</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>4.071464856465657</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>3.941786766052246</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>2.862774610519409</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>